<commit_message>
refactor: update notebook analysis, reorganize mappings, and synchronize exports with new heatmap and performance plots
</commit_message>
<xml_diff>
--- a/exports/NursIT_Allgemeine_Verbandsklassen.xlsx
+++ b/exports/NursIT_Allgemeine_Verbandsklassen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mertakdemir/Developer/uni/Modell/exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2142C364-ED42-A34F-B53C-C8161897DB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8326259D-6808-444E-9BC1-D97190F667FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35060" windowHeight="27800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NursIT Experte" sheetId="2" r:id="rId1"/>
@@ -4239,21 +4239,25 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0F172A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -14890,6 +14894,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -26922,6 +26927,18 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A57:A59"/>
+    <mergeCell ref="A33:A35"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A42:A44"/>
@@ -26931,20 +26948,9 @@
     <mergeCell ref="A36:A38"/>
     <mergeCell ref="A30:A32"/>
     <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A57:A59"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A63:A65"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="A54:A56"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -26954,7 +26960,7 @@
   <dimension ref="A1:BJ86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="62" width="36" customWidth="1"/>
   </cols>
@@ -42883,12 +42889,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A83:A86"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="A51:A54"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="A55:A58"/>
     <mergeCell ref="A71:A74"/>
@@ -42900,12 +42900,19 @@
     <mergeCell ref="A31:A34"/>
     <mergeCell ref="A43:A46"/>
     <mergeCell ref="A67:A70"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A83:A86"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A51:A54"/>
     <mergeCell ref="A79:A82"/>
-    <mergeCell ref="A11:A14"/>
     <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A7:A10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>